<commit_message>
Fix Indonesia input path and include Nariño temperatures (#5)
</commit_message>
<xml_diff>
--- a/data/clean/temp/Colombia_temp.xlsx
+++ b/data/clean/temp/Colombia_temp.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P131"/>
+  <dimension ref="A1:P157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4874,52 +4874,52 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>2000</v>
       </c>
       <c r="E80" t="n">
-        <v>17.02</v>
+        <v>20.04</v>
       </c>
       <c r="F80" t="n">
-        <v>17.17</v>
+        <v>20.24</v>
       </c>
       <c r="G80" t="n">
-        <v>17.33</v>
+        <v>20.5</v>
       </c>
       <c r="H80" t="n">
-        <v>17.65</v>
+        <v>20.88</v>
       </c>
       <c r="I80" t="n">
-        <v>17.43</v>
+        <v>20.59</v>
       </c>
       <c r="J80" t="n">
-        <v>17.29</v>
+        <v>20.4</v>
       </c>
       <c r="K80" t="n">
-        <v>17.16</v>
+        <v>20.22</v>
       </c>
       <c r="L80" t="n">
-        <v>17.78</v>
+        <v>21.03</v>
       </c>
       <c r="M80" t="n">
-        <v>17.2</v>
+        <v>20.33</v>
       </c>
       <c r="N80" t="n">
-        <v>17.74</v>
+        <v>21.16</v>
       </c>
       <c r="O80" t="n">
-        <v>17.41</v>
+        <v>20.59</v>
       </c>
       <c r="P80" t="n">
-        <v>17.68</v>
+        <v>20.57</v>
       </c>
     </row>
     <row r="81">
@@ -4930,52 +4930,52 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D81" t="n">
         <v>2001</v>
       </c>
       <c r="E81" t="n">
-        <v>17.36</v>
+        <v>20.6</v>
       </c>
       <c r="F81" t="n">
-        <v>17.6</v>
+        <v>21.22</v>
       </c>
       <c r="G81" t="n">
-        <v>17.73</v>
+        <v>21.25</v>
       </c>
       <c r="H81" t="n">
-        <v>18.09</v>
+        <v>21.55</v>
       </c>
       <c r="I81" t="n">
-        <v>17.81</v>
+        <v>20.93</v>
       </c>
       <c r="J81" t="n">
-        <v>17.5</v>
+        <v>20.52</v>
       </c>
       <c r="K81" t="n">
-        <v>17.72</v>
+        <v>20.69</v>
       </c>
       <c r="L81" t="n">
-        <v>18.71</v>
+        <v>21.34</v>
       </c>
       <c r="M81" t="n">
-        <v>17.84</v>
+        <v>20.71</v>
       </c>
       <c r="N81" t="n">
-        <v>17.99</v>
+        <v>21.29</v>
       </c>
       <c r="O81" t="n">
-        <v>17.75</v>
+        <v>21.01</v>
       </c>
       <c r="P81" t="n">
-        <v>17.96</v>
+        <v>21.11</v>
       </c>
     </row>
     <row r="82">
@@ -4986,52 +4986,52 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D82" t="n">
         <v>2002</v>
       </c>
       <c r="E82" t="n">
-        <v>18.16</v>
+        <v>20.99</v>
       </c>
       <c r="F82" t="n">
-        <v>18.21</v>
+        <v>21.71</v>
       </c>
       <c r="G82" t="n">
-        <v>18.02</v>
+        <v>21.65</v>
       </c>
       <c r="H82" t="n">
-        <v>17.75</v>
+        <v>21.55</v>
       </c>
       <c r="I82" t="n">
-        <v>18.16</v>
+        <v>21.73</v>
       </c>
       <c r="J82" t="n">
-        <v>17.42</v>
+        <v>20.71</v>
       </c>
       <c r="K82" t="n">
-        <v>18.02</v>
+        <v>21.06</v>
       </c>
       <c r="L82" t="n">
-        <v>18.32</v>
+        <v>21.22</v>
       </c>
       <c r="M82" t="n">
-        <v>18.24</v>
+        <v>21.33</v>
       </c>
       <c r="N82" t="n">
-        <v>17.9</v>
+        <v>21.48</v>
       </c>
       <c r="O82" t="n">
-        <v>17.95</v>
+        <v>21.39</v>
       </c>
       <c r="P82" t="n">
-        <v>18.49</v>
+        <v>21.61</v>
       </c>
     </row>
     <row r="83">
@@ -5042,52 +5042,52 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D83" t="n">
         <v>2003</v>
       </c>
       <c r="E83" t="n">
-        <v>18.55</v>
+        <v>21.63</v>
       </c>
       <c r="F83" t="n">
-        <v>18.72</v>
+        <v>21.81</v>
       </c>
       <c r="G83" t="n">
-        <v>18.37</v>
+        <v>21.65</v>
       </c>
       <c r="H83" t="n">
-        <v>18.31</v>
+        <v>21.58</v>
       </c>
       <c r="I83" t="n">
-        <v>18.3</v>
+        <v>21.53</v>
       </c>
       <c r="J83" t="n">
-        <v>17.21</v>
+        <v>20.68</v>
       </c>
       <c r="K83" t="n">
-        <v>17.62</v>
+        <v>20.87</v>
       </c>
       <c r="L83" t="n">
-        <v>17.82</v>
+        <v>20.77</v>
       </c>
       <c r="M83" t="n">
-        <v>17.88</v>
+        <v>20.97</v>
       </c>
       <c r="N83" t="n">
-        <v>17.55</v>
+        <v>21.24</v>
       </c>
       <c r="O83" t="n">
-        <v>17.56</v>
+        <v>20.91</v>
       </c>
       <c r="P83" t="n">
-        <v>17.84</v>
+        <v>21.07</v>
       </c>
     </row>
     <row r="84">
@@ -5098,52 +5098,52 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D84" t="n">
         <v>2004</v>
       </c>
       <c r="E84" t="n">
-        <v>17.61</v>
+        <v>20.89</v>
       </c>
       <c r="F84" t="n">
-        <v>18.2</v>
+        <v>21.51</v>
       </c>
       <c r="G84" t="n">
-        <v>18.76</v>
+        <v>22.17</v>
       </c>
       <c r="H84" t="n">
-        <v>18.09</v>
+        <v>21.55</v>
       </c>
       <c r="I84" t="n">
-        <v>17.7</v>
+        <v>20.96</v>
       </c>
       <c r="J84" t="n">
-        <v>17.92</v>
+        <v>21</v>
       </c>
       <c r="K84" t="n">
-        <v>17.37</v>
+        <v>20.53</v>
       </c>
       <c r="L84" t="n">
-        <v>18.16</v>
+        <v>20.98</v>
       </c>
       <c r="M84" t="n">
-        <v>17.28</v>
+        <v>20.83</v>
       </c>
       <c r="N84" t="n">
-        <v>17.35</v>
+        <v>21.06</v>
       </c>
       <c r="O84" t="n">
-        <v>17.45</v>
+        <v>21.1</v>
       </c>
       <c r="P84" t="n">
-        <v>17.64</v>
+        <v>21.13</v>
       </c>
     </row>
     <row r="85">
@@ -5154,52 +5154,52 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D85" t="n">
         <v>2005</v>
       </c>
       <c r="E85" t="n">
-        <v>17.82</v>
+        <v>21.1</v>
       </c>
       <c r="F85" t="n">
-        <v>18.21</v>
+        <v>21.37</v>
       </c>
       <c r="G85" t="n">
-        <v>18.57</v>
+        <v>21.56</v>
       </c>
       <c r="H85" t="n">
-        <v>18.8</v>
+        <v>22.01</v>
       </c>
       <c r="I85" t="n">
-        <v>17.95</v>
+        <v>21.3</v>
       </c>
       <c r="J85" t="n">
-        <v>18.05</v>
+        <v>21.2</v>
       </c>
       <c r="K85" t="n">
-        <v>18.26</v>
+        <v>21.23</v>
       </c>
       <c r="L85" t="n">
-        <v>18.22</v>
+        <v>21.24</v>
       </c>
       <c r="M85" t="n">
-        <v>18.23</v>
+        <v>21.12</v>
       </c>
       <c r="N85" t="n">
-        <v>17.3</v>
+        <v>20.55</v>
       </c>
       <c r="O85" t="n">
-        <v>17.35</v>
+        <v>20.35</v>
       </c>
       <c r="P85" t="n">
-        <v>17.25</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="86">
@@ -5210,52 +5210,52 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D86" t="n">
         <v>2006</v>
       </c>
       <c r="E86" t="n">
-        <v>17.63</v>
+        <v>20.79</v>
       </c>
       <c r="F86" t="n">
-        <v>18.11</v>
+        <v>21.46</v>
       </c>
       <c r="G86" t="n">
-        <v>17.72</v>
+        <v>21.11</v>
       </c>
       <c r="H86" t="n">
-        <v>17.89</v>
+        <v>21.07</v>
       </c>
       <c r="I86" t="n">
-        <v>17.84</v>
+        <v>21.18</v>
       </c>
       <c r="J86" t="n">
-        <v>17.61</v>
+        <v>20.94</v>
       </c>
       <c r="K86" t="n">
-        <v>18.12</v>
+        <v>21.35</v>
       </c>
       <c r="L86" t="n">
-        <v>18.22</v>
+        <v>21.35</v>
       </c>
       <c r="M86" t="n">
-        <v>18.14</v>
+        <v>21.49</v>
       </c>
       <c r="N86" t="n">
-        <v>18.09</v>
+        <v>21.46</v>
       </c>
       <c r="O86" t="n">
-        <v>17.76</v>
+        <v>20.98</v>
       </c>
       <c r="P86" t="n">
-        <v>17.94</v>
+        <v>21.08</v>
       </c>
     </row>
     <row r="87">
@@ -5266,52 +5266,52 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D87" t="n">
         <v>2007</v>
       </c>
       <c r="E87" t="n">
-        <v>18.01</v>
+        <v>21.57</v>
       </c>
       <c r="F87" t="n">
-        <v>18.44</v>
+        <v>21.41</v>
       </c>
       <c r="G87" t="n">
-        <v>18.17</v>
+        <v>21.3</v>
       </c>
       <c r="H87" t="n">
-        <v>17.95</v>
+        <v>21.18</v>
       </c>
       <c r="I87" t="n">
-        <v>17.8</v>
+        <v>20.92</v>
       </c>
       <c r="J87" t="n">
-        <v>17.7</v>
+        <v>20.48</v>
       </c>
       <c r="K87" t="n">
-        <v>17.92</v>
+        <v>20.75</v>
       </c>
       <c r="L87" t="n">
-        <v>17.48</v>
+        <v>20.25</v>
       </c>
       <c r="M87" t="n">
-        <v>17.77</v>
+        <v>20.76</v>
       </c>
       <c r="N87" t="n">
-        <v>17</v>
+        <v>20.29</v>
       </c>
       <c r="O87" t="n">
-        <v>17.21</v>
+        <v>20.38</v>
       </c>
       <c r="P87" t="n">
-        <v>17.49</v>
+        <v>20.11</v>
       </c>
     </row>
     <row r="88">
@@ -5322,52 +5322,52 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D88" t="n">
         <v>2008</v>
       </c>
       <c r="E88" t="n">
-        <v>17.52</v>
+        <v>20.64</v>
       </c>
       <c r="F88" t="n">
-        <v>17.62</v>
+        <v>20.89</v>
       </c>
       <c r="G88" t="n">
-        <v>17.52</v>
+        <v>21.1</v>
       </c>
       <c r="H88" t="n">
-        <v>17.74</v>
+        <v>20.97</v>
       </c>
       <c r="I88" t="n">
-        <v>17.25</v>
+        <v>20.51</v>
       </c>
       <c r="J88" t="n">
-        <v>17.45</v>
+        <v>20.72</v>
       </c>
       <c r="K88" t="n">
-        <v>17.32</v>
+        <v>20.75</v>
       </c>
       <c r="L88" t="n">
-        <v>17.34</v>
+        <v>20.69</v>
       </c>
       <c r="M88" t="n">
-        <v>17.69</v>
+        <v>20.99</v>
       </c>
       <c r="N88" t="n">
-        <v>17.39</v>
+        <v>20.77</v>
       </c>
       <c r="O88" t="n">
-        <v>17.35</v>
+        <v>20.59</v>
       </c>
       <c r="P88" t="n">
-        <v>17.28</v>
+        <v>20.48</v>
       </c>
     </row>
     <row r="89">
@@ -5378,52 +5378,52 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D89" t="n">
         <v>2009</v>
       </c>
       <c r="E89" t="n">
-        <v>17.62</v>
+        <v>20.58</v>
       </c>
       <c r="F89" t="n">
-        <v>17.59</v>
+        <v>20.93</v>
       </c>
       <c r="G89" t="n">
-        <v>16.98</v>
+        <v>20.2</v>
       </c>
       <c r="H89" t="n">
-        <v>18.39</v>
+        <v>21.56</v>
       </c>
       <c r="I89" t="n">
-        <v>18.15</v>
+        <v>21.5</v>
       </c>
       <c r="J89" t="n">
-        <v>18.13</v>
+        <v>21.43</v>
       </c>
       <c r="K89" t="n">
-        <v>18.53</v>
+        <v>21.67</v>
       </c>
       <c r="L89" t="n">
-        <v>18.84</v>
+        <v>21.83</v>
       </c>
       <c r="M89" t="n">
-        <v>19.02</v>
+        <v>21.94</v>
       </c>
       <c r="N89" t="n">
-        <v>18.38</v>
+        <v>21.64</v>
       </c>
       <c r="O89" t="n">
-        <v>18.62</v>
+        <v>21.73</v>
       </c>
       <c r="P89" t="n">
-        <v>18.46</v>
+        <v>21.68</v>
       </c>
     </row>
     <row r="90">
@@ -5434,52 +5434,52 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D90" t="n">
         <v>2010</v>
       </c>
       <c r="E90" t="n">
-        <v>18.81</v>
+        <v>21.88</v>
       </c>
       <c r="F90" t="n">
-        <v>18.96</v>
+        <v>22.06</v>
       </c>
       <c r="G90" t="n">
-        <v>19.61</v>
+        <v>22.47</v>
       </c>
       <c r="H90" t="n">
-        <v>18.71</v>
+        <v>21.97</v>
       </c>
       <c r="I90" t="n">
-        <v>18.51</v>
+        <v>21.8</v>
       </c>
       <c r="J90" t="n">
-        <v>17.87</v>
+        <v>21.11</v>
       </c>
       <c r="K90" t="n">
-        <v>17.66</v>
+        <v>20.7</v>
       </c>
       <c r="L90" t="n">
-        <v>17.99</v>
+        <v>20.77</v>
       </c>
       <c r="M90" t="n">
-        <v>17.71</v>
+        <v>20.64</v>
       </c>
       <c r="N90" t="n">
-        <v>17.75</v>
+        <v>20.76</v>
       </c>
       <c r="O90" t="n">
-        <v>17.09</v>
+        <v>20.22</v>
       </c>
       <c r="P90" t="n">
-        <v>17.09</v>
+        <v>20.05</v>
       </c>
     </row>
     <row r="91">
@@ -5490,52 +5490,52 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D91" t="n">
         <v>2011</v>
       </c>
       <c r="E91" t="n">
-        <v>17.72</v>
+        <v>20.63</v>
       </c>
       <c r="F91" t="n">
-        <v>17.66</v>
+        <v>20.69</v>
       </c>
       <c r="G91" t="n">
-        <v>17.43</v>
+        <v>20.66</v>
       </c>
       <c r="H91" t="n">
-        <v>17.62</v>
+        <v>21.14</v>
       </c>
       <c r="I91" t="n">
-        <v>17.91</v>
+        <v>21.46</v>
       </c>
       <c r="J91" t="n">
-        <v>18.26</v>
+        <v>21.69</v>
       </c>
       <c r="K91" t="n">
-        <v>18.03</v>
+        <v>21.12</v>
       </c>
       <c r="L91" t="n">
-        <v>18.28</v>
+        <v>21.33</v>
       </c>
       <c r="M91" t="n">
-        <v>18.33</v>
+        <v>21.24</v>
       </c>
       <c r="N91" t="n">
-        <v>17.21</v>
+        <v>20.43</v>
       </c>
       <c r="O91" t="n">
-        <v>17.66</v>
+        <v>20.89</v>
       </c>
       <c r="P91" t="n">
-        <v>17.46</v>
+        <v>20.83</v>
       </c>
     </row>
     <row r="92">
@@ -5546,52 +5546,52 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D92" t="n">
         <v>2012</v>
       </c>
       <c r="E92" t="n">
-        <v>17.58</v>
+        <v>20.63</v>
       </c>
       <c r="F92" t="n">
-        <v>17.82</v>
+        <v>20.69</v>
       </c>
       <c r="G92" t="n">
-        <v>18.12</v>
+        <v>21.4</v>
       </c>
       <c r="H92" t="n">
-        <v>17.8</v>
+        <v>21.44</v>
       </c>
       <c r="I92" t="n">
-        <v>18.21</v>
+        <v>21.67</v>
       </c>
       <c r="J92" t="n">
-        <v>18.4</v>
+        <v>21.83</v>
       </c>
       <c r="K92" t="n">
-        <v>18.57</v>
+        <v>21.68</v>
       </c>
       <c r="L92" t="n">
-        <v>18.32</v>
+        <v>21.33</v>
       </c>
       <c r="M92" t="n">
-        <v>18.77</v>
+        <v>21.6</v>
       </c>
       <c r="N92" t="n">
-        <v>18.1</v>
+        <v>21.27</v>
       </c>
       <c r="O92" t="n">
-        <v>17.9</v>
+        <v>21.2</v>
       </c>
       <c r="P92" t="n">
-        <v>18.28</v>
+        <v>21.11</v>
       </c>
     </row>
     <row r="93">
@@ -5602,52 +5602,52 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D93" t="n">
         <v>2013</v>
       </c>
       <c r="E93" t="n">
-        <v>18.9</v>
+        <v>21.54</v>
       </c>
       <c r="F93" t="n">
-        <v>18.26</v>
+        <v>21.27</v>
       </c>
       <c r="G93" t="n">
-        <v>18.72</v>
+        <v>21.6</v>
       </c>
       <c r="H93" t="n">
-        <v>18.9</v>
+        <v>21.44</v>
       </c>
       <c r="I93" t="n">
-        <v>17.72</v>
+        <v>21</v>
       </c>
       <c r="J93" t="n">
-        <v>18.51</v>
+        <v>21.19</v>
       </c>
       <c r="K93" t="n">
-        <v>18.37</v>
+        <v>21.07</v>
       </c>
       <c r="L93" t="n">
-        <v>18.03</v>
+        <v>20.88</v>
       </c>
       <c r="M93" t="n">
-        <v>18.64</v>
+        <v>21.45</v>
       </c>
       <c r="N93" t="n">
-        <v>18.29</v>
+        <v>21.21</v>
       </c>
       <c r="O93" t="n">
-        <v>18.02</v>
+        <v>21.11</v>
       </c>
       <c r="P93" t="n">
-        <v>18.04</v>
+        <v>21.12</v>
       </c>
     </row>
     <row r="94">
@@ -5658,52 +5658,52 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D94" t="n">
         <v>2014</v>
       </c>
       <c r="E94" t="n">
-        <v>18.32</v>
+        <v>21.37</v>
       </c>
       <c r="F94" t="n">
-        <v>18.41</v>
+        <v>21.36</v>
       </c>
       <c r="G94" t="n">
-        <v>18.47</v>
+        <v>21.61</v>
       </c>
       <c r="H94" t="n">
-        <v>18.94</v>
+        <v>21.86</v>
       </c>
       <c r="I94" t="n">
-        <v>18.31</v>
+        <v>21.87</v>
       </c>
       <c r="J94" t="n">
-        <v>18.8</v>
+        <v>22.15</v>
       </c>
       <c r="K94" t="n">
-        <v>19.41</v>
+        <v>22.12</v>
       </c>
       <c r="L94" t="n">
-        <v>18.82</v>
+        <v>21.59</v>
       </c>
       <c r="M94" t="n">
-        <v>18.83</v>
+        <v>21.76</v>
       </c>
       <c r="N94" t="n">
-        <v>18.2</v>
+        <v>21.64</v>
       </c>
       <c r="O94" t="n">
-        <v>18.35</v>
+        <v>21.53</v>
       </c>
       <c r="P94" t="n">
-        <v>18.53</v>
+        <v>21.53</v>
       </c>
     </row>
     <row r="95">
@@ -5714,52 +5714,52 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D95" t="n">
         <v>2015</v>
       </c>
       <c r="E95" t="n">
-        <v>18.66</v>
+        <v>21.54</v>
       </c>
       <c r="F95" t="n">
-        <v>18.81</v>
+        <v>21.82</v>
       </c>
       <c r="G95" t="n">
-        <v>18.43</v>
+        <v>21.78</v>
       </c>
       <c r="H95" t="n">
-        <v>18.7</v>
+        <v>22.04</v>
       </c>
       <c r="I95" t="n">
-        <v>19.02</v>
+        <v>22.52</v>
       </c>
       <c r="J95" t="n">
-        <v>18.7</v>
+        <v>22.31</v>
       </c>
       <c r="K95" t="n">
-        <v>19.04</v>
+        <v>22.23</v>
       </c>
       <c r="L95" t="n">
-        <v>19.32</v>
+        <v>22.26</v>
       </c>
       <c r="M95" t="n">
-        <v>19.38</v>
+        <v>22.62</v>
       </c>
       <c r="N95" t="n">
-        <v>18.89</v>
+        <v>22.36</v>
       </c>
       <c r="O95" t="n">
-        <v>18.62</v>
+        <v>22.1</v>
       </c>
       <c r="P95" t="n">
-        <v>18.93</v>
+        <v>22.37</v>
       </c>
     </row>
     <row r="96">
@@ -5770,52 +5770,52 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D96" t="n">
         <v>2016</v>
       </c>
       <c r="E96" t="n">
-        <v>19.21</v>
+        <v>22.44</v>
       </c>
       <c r="F96" t="n">
-        <v>19.41</v>
+        <v>22.57</v>
       </c>
       <c r="G96" t="n">
-        <v>18.78</v>
+        <v>22.23</v>
       </c>
       <c r="H96" t="n">
-        <v>19.11</v>
+        <v>22.24</v>
       </c>
       <c r="I96" t="n">
-        <v>19.05</v>
+        <v>22.33</v>
       </c>
       <c r="J96" t="n">
-        <v>18.56</v>
+        <v>21.79</v>
       </c>
       <c r="K96" t="n">
-        <v>18.48</v>
+        <v>21.59</v>
       </c>
       <c r="L96" t="n">
-        <v>19.24</v>
+        <v>22.05</v>
       </c>
       <c r="M96" t="n">
-        <v>18.44</v>
+        <v>21.7</v>
       </c>
       <c r="N96" t="n">
-        <v>18.11</v>
+        <v>21.6</v>
       </c>
       <c r="O96" t="n">
-        <v>17.88</v>
+        <v>21.29</v>
       </c>
       <c r="P96" t="n">
-        <v>17.9</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="97">
@@ -5826,52 +5826,52 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D97" t="n">
         <v>2017</v>
       </c>
       <c r="E97" t="n">
-        <v>17.71</v>
+        <v>21.16</v>
       </c>
       <c r="F97" t="n">
-        <v>18.21</v>
+        <v>21.5</v>
       </c>
       <c r="G97" t="n">
-        <v>17.72</v>
+        <v>21.38</v>
       </c>
       <c r="H97" t="n">
-        <v>18.69</v>
+        <v>21.91</v>
       </c>
       <c r="I97" t="n">
-        <v>18.21</v>
+        <v>21.69</v>
       </c>
       <c r="J97" t="n">
-        <v>18.07</v>
+        <v>21.37</v>
       </c>
       <c r="K97" t="n">
-        <v>18.42</v>
+        <v>21.51</v>
       </c>
       <c r="L97" t="n">
-        <v>18.01</v>
+        <v>21.42</v>
       </c>
       <c r="M97" t="n">
-        <v>18.77</v>
+        <v>21.76</v>
       </c>
       <c r="N97" t="n">
-        <v>18.14</v>
+        <v>21.88</v>
       </c>
       <c r="O97" t="n">
-        <v>18.05</v>
+        <v>21.23</v>
       </c>
       <c r="P97" t="n">
-        <v>17.78</v>
+        <v>20.82</v>
       </c>
     </row>
     <row r="98">
@@ -5882,52 +5882,52 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D98" t="n">
         <v>2018</v>
       </c>
       <c r="E98" t="n">
-        <v>17.71</v>
+        <v>20.95</v>
       </c>
       <c r="F98" t="n">
-        <v>18.01</v>
+        <v>21.19</v>
       </c>
       <c r="G98" t="n">
-        <v>18.47</v>
+        <v>21.67</v>
       </c>
       <c r="H98" t="n">
-        <v>17.89</v>
+        <v>21.36</v>
       </c>
       <c r="I98" t="n">
-        <v>17.75</v>
+        <v>22.05</v>
       </c>
       <c r="J98" t="n">
-        <v>18.1</v>
+        <v>21.58</v>
       </c>
       <c r="K98" t="n">
-        <v>18.22</v>
+        <v>21.6</v>
       </c>
       <c r="L98" t="n">
-        <v>18.42</v>
+        <v>21.61</v>
       </c>
       <c r="M98" t="n">
-        <v>18.33</v>
+        <v>21.68</v>
       </c>
       <c r="N98" t="n">
-        <v>17.9</v>
+        <v>21.64</v>
       </c>
       <c r="O98" t="n">
-        <v>17.96</v>
+        <v>21.48</v>
       </c>
       <c r="P98" t="n">
-        <v>18.32</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="99">
@@ -5938,52 +5938,52 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D99" t="n">
         <v>2019</v>
       </c>
       <c r="E99" t="n">
-        <v>18.41</v>
+        <v>21.64</v>
       </c>
       <c r="F99" t="n">
-        <v>18.91</v>
+        <v>21.99</v>
       </c>
       <c r="G99" t="n">
-        <v>18.42</v>
+        <v>21.75</v>
       </c>
       <c r="H99" t="n">
-        <v>18.7</v>
+        <v>21.95</v>
       </c>
       <c r="I99" t="n">
-        <v>18.31</v>
+        <v>21.9</v>
       </c>
       <c r="J99" t="n">
-        <v>18.65</v>
+        <v>21.92</v>
       </c>
       <c r="K99" t="n">
-        <v>18.66</v>
+        <v>21.84</v>
       </c>
       <c r="L99" t="n">
-        <v>19.11</v>
+        <v>21.74</v>
       </c>
       <c r="M99" t="n">
-        <v>18.83</v>
+        <v>21.69</v>
       </c>
       <c r="N99" t="n">
-        <v>17.89</v>
+        <v>21.19</v>
       </c>
       <c r="O99" t="n">
-        <v>18.3</v>
+        <v>21.54</v>
       </c>
       <c r="P99" t="n">
-        <v>18.43</v>
+        <v>21.67</v>
       </c>
     </row>
     <row r="100">
@@ -5994,52 +5994,52 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D100" t="n">
         <v>2020</v>
       </c>
       <c r="E100" t="n">
-        <v>18.8</v>
+        <v>21.8</v>
       </c>
       <c r="F100" t="n">
-        <v>19.34</v>
+        <v>22.36</v>
       </c>
       <c r="G100" t="n">
-        <v>19.06</v>
+        <v>22.36</v>
       </c>
       <c r="H100" t="n">
-        <v>19.09</v>
+        <v>22.39</v>
       </c>
       <c r="I100" t="n">
-        <v>18.54</v>
+        <v>21.92</v>
       </c>
       <c r="J100" t="n">
-        <v>18.15</v>
+        <v>21.76</v>
       </c>
       <c r="K100" t="n">
-        <v>18.02</v>
+        <v>21.67</v>
       </c>
       <c r="L100" t="n">
-        <v>18.12</v>
+        <v>21.47</v>
       </c>
       <c r="M100" t="n">
-        <v>18.09</v>
+        <v>21.39</v>
       </c>
       <c r="N100" t="n">
-        <v>18.09</v>
+        <v>21.61</v>
       </c>
       <c r="O100" t="n">
-        <v>17.75</v>
+        <v>21.1</v>
       </c>
       <c r="P100" t="n">
-        <v>17.83</v>
+        <v>20.95</v>
       </c>
     </row>
     <row r="101">
@@ -6050,52 +6050,52 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D101" t="n">
         <v>2021</v>
       </c>
       <c r="E101" t="n">
-        <v>18.04</v>
+        <v>21.25</v>
       </c>
       <c r="F101" t="n">
-        <v>18.16</v>
+        <v>20.69</v>
       </c>
       <c r="G101" t="n">
-        <v>17.42</v>
+        <v>20.64</v>
       </c>
       <c r="H101" t="n">
-        <v>18.1</v>
+        <v>21.51</v>
       </c>
       <c r="I101" t="n">
-        <v>18</v>
+        <v>21.48</v>
       </c>
       <c r="J101" t="n">
-        <v>17.41</v>
+        <v>21.04</v>
       </c>
       <c r="K101" t="n">
-        <v>18.02</v>
+        <v>21.7</v>
       </c>
       <c r="L101" t="n">
-        <v>17.43</v>
+        <v>21.27</v>
       </c>
       <c r="M101" t="n">
-        <v>17.93</v>
+        <v>21.33</v>
       </c>
       <c r="N101" t="n">
-        <v>17.7</v>
+        <v>21.45</v>
       </c>
       <c r="O101" t="n">
-        <v>17.56</v>
+        <v>21.16</v>
       </c>
       <c r="P101" t="n">
-        <v>17.85</v>
+        <v>21.34</v>
       </c>
     </row>
     <row r="102">
@@ -6106,52 +6106,52 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D102" t="n">
         <v>2022</v>
       </c>
       <c r="E102" t="n">
-        <v>17.72</v>
+        <v>21.11</v>
       </c>
       <c r="F102" t="n">
-        <v>17.57</v>
+        <v>20.96</v>
       </c>
       <c r="G102" t="n">
-        <v>17.47</v>
+        <v>20.9</v>
       </c>
       <c r="H102" t="n">
-        <v>17.9</v>
+        <v>21.09</v>
       </c>
       <c r="I102" t="n">
-        <v>17.9</v>
+        <v>21.23</v>
       </c>
       <c r="J102" t="n">
-        <v>16.61</v>
+        <v>20.18</v>
       </c>
       <c r="K102" t="n">
-        <v>17.52</v>
+        <v>20.87</v>
       </c>
       <c r="L102" t="n">
-        <v>17.68</v>
+        <v>20.84</v>
       </c>
       <c r="M102" t="n">
-        <v>17.53</v>
+        <v>20.95</v>
       </c>
       <c r="N102" t="n">
-        <v>17.74</v>
+        <v>21.22</v>
       </c>
       <c r="O102" t="n">
-        <v>17.21</v>
+        <v>20.83</v>
       </c>
       <c r="P102" t="n">
-        <v>17.43</v>
+        <v>21.13</v>
       </c>
     </row>
     <row r="103">
@@ -6162,52 +6162,52 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D103" t="n">
         <v>2023</v>
       </c>
       <c r="E103" t="n">
-        <v>17.22</v>
+        <v>20.53</v>
       </c>
       <c r="F103" t="n">
-        <v>18.11</v>
+        <v>21.56</v>
       </c>
       <c r="G103" t="n">
-        <v>17.57</v>
+        <v>21.37</v>
       </c>
       <c r="H103" t="n">
-        <v>17.9</v>
+        <v>21.9</v>
       </c>
       <c r="I103" t="n">
-        <v>18.61</v>
+        <v>22.52</v>
       </c>
       <c r="J103" t="n">
-        <v>18.57</v>
+        <v>22.38</v>
       </c>
       <c r="K103" t="n">
-        <v>18.62</v>
+        <v>22.33</v>
       </c>
       <c r="L103" t="n">
-        <v>18.82</v>
+        <v>22.37</v>
       </c>
       <c r="M103" t="n">
-        <v>18.87</v>
+        <v>22.36</v>
       </c>
       <c r="N103" t="n">
-        <v>18.44</v>
+        <v>22.21</v>
       </c>
       <c r="O103" t="n">
-        <v>18.35</v>
+        <v>21.94</v>
       </c>
       <c r="P103" t="n">
-        <v>18.48</v>
+        <v>21.72</v>
       </c>
     </row>
     <row r="104">
@@ -6218,52 +6218,52 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>2024</v>
       </c>
       <c r="E104" t="n">
-        <v>19.06</v>
+        <v>22.17</v>
       </c>
       <c r="F104" t="n">
-        <v>19.5</v>
+        <v>22.53</v>
       </c>
       <c r="G104" t="n">
-        <v>18.81</v>
+        <v>22.15</v>
       </c>
       <c r="H104" t="n">
-        <v>19</v>
+        <v>22.22</v>
       </c>
       <c r="I104" t="n">
-        <v>18.85</v>
+        <v>21.94</v>
       </c>
       <c r="J104" t="n">
-        <v>17.81</v>
+        <v>21.2</v>
       </c>
       <c r="K104" t="n">
-        <v>18.77</v>
+        <v>21.82</v>
       </c>
       <c r="L104" t="n">
-        <v>18.77</v>
+        <v>21.77</v>
       </c>
       <c r="M104" t="n">
-        <v>19.24</v>
+        <v>22.31</v>
       </c>
       <c r="N104" t="n">
-        <v>18.19</v>
+        <v>21.55</v>
       </c>
       <c r="O104" t="n">
-        <v>18.02</v>
+        <v>21.45</v>
       </c>
       <c r="P104" t="n">
-        <v>18.39</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="105">
@@ -6274,52 +6274,52 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>COL.57958</t>
+          <t>COL.57955</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Quindio</t>
+          <t>Nariño</t>
         </is>
       </c>
       <c r="D105" t="n">
         <v>2025</v>
       </c>
       <c r="E105" t="n">
-        <v>18.41</v>
+        <v>21.34</v>
       </c>
       <c r="F105" t="n">
-        <v>18.12</v>
+        <v>21.35</v>
       </c>
       <c r="G105" t="n">
-        <v>18.42</v>
+        <v>21.61</v>
       </c>
       <c r="H105" t="n">
-        <v>18.8</v>
+        <v>22.03</v>
       </c>
       <c r="I105" t="n">
-        <v>18.6</v>
+        <v>21.89</v>
       </c>
       <c r="J105" t="n">
-        <v>18.01</v>
+        <v>21.59</v>
       </c>
       <c r="K105" t="n">
-        <v>18.96</v>
+        <v>22</v>
       </c>
       <c r="L105" t="n">
-        <v>18.72</v>
+        <v>21.7</v>
       </c>
       <c r="M105" t="n">
-        <v>18.84</v>
+        <v>21.98</v>
       </c>
       <c r="N105" t="n">
-        <v>18.2</v>
+        <v>21.63</v>
       </c>
       <c r="O105" t="n">
-        <v>18.55</v>
+        <v>21.57</v>
       </c>
       <c r="P105" t="n">
-        <v>18.33</v>
+        <v>21.36</v>
       </c>
     </row>
     <row r="106">
@@ -6330,52 +6330,52 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D106" t="n">
         <v>2000</v>
       </c>
       <c r="E106" t="n">
-        <v>19.75</v>
+        <v>17.02</v>
       </c>
       <c r="F106" t="n">
-        <v>19.95</v>
+        <v>17.17</v>
       </c>
       <c r="G106" t="n">
-        <v>20.09</v>
+        <v>17.33</v>
       </c>
       <c r="H106" t="n">
-        <v>20.27</v>
+        <v>17.65</v>
       </c>
       <c r="I106" t="n">
-        <v>20.03</v>
+        <v>17.43</v>
       </c>
       <c r="J106" t="n">
-        <v>19.83</v>
+        <v>17.29</v>
       </c>
       <c r="K106" t="n">
-        <v>19.85</v>
+        <v>17.16</v>
       </c>
       <c r="L106" t="n">
-        <v>20.36</v>
+        <v>17.78</v>
       </c>
       <c r="M106" t="n">
-        <v>19.81</v>
+        <v>17.2</v>
       </c>
       <c r="N106" t="n">
-        <v>20.19</v>
+        <v>17.74</v>
       </c>
       <c r="O106" t="n">
-        <v>19.81</v>
+        <v>17.41</v>
       </c>
       <c r="P106" t="n">
-        <v>20.19</v>
+        <v>17.68</v>
       </c>
     </row>
     <row r="107">
@@ -6386,52 +6386,52 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D107" t="n">
         <v>2001</v>
       </c>
       <c r="E107" t="n">
-        <v>20.22</v>
+        <v>17.36</v>
       </c>
       <c r="F107" t="n">
-        <v>20.16</v>
+        <v>17.6</v>
       </c>
       <c r="G107" t="n">
-        <v>20.61</v>
+        <v>17.73</v>
       </c>
       <c r="H107" t="n">
-        <v>20.54</v>
+        <v>18.09</v>
       </c>
       <c r="I107" t="n">
-        <v>20.55</v>
+        <v>17.81</v>
       </c>
       <c r="J107" t="n">
-        <v>20.18</v>
+        <v>17.5</v>
       </c>
       <c r="K107" t="n">
-        <v>20.59</v>
+        <v>17.72</v>
       </c>
       <c r="L107" t="n">
-        <v>21.21</v>
+        <v>18.71</v>
       </c>
       <c r="M107" t="n">
-        <v>20.54</v>
+        <v>17.84</v>
       </c>
       <c r="N107" t="n">
-        <v>20.44</v>
+        <v>17.99</v>
       </c>
       <c r="O107" t="n">
-        <v>20.28</v>
+        <v>17.75</v>
       </c>
       <c r="P107" t="n">
-        <v>20.71</v>
+        <v>17.96</v>
       </c>
     </row>
     <row r="108">
@@ -6442,52 +6442,52 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D108" t="n">
         <v>2002</v>
       </c>
       <c r="E108" t="n">
-        <v>20.86</v>
+        <v>18.16</v>
       </c>
       <c r="F108" t="n">
-        <v>20.77</v>
+        <v>18.21</v>
       </c>
       <c r="G108" t="n">
-        <v>20.73</v>
+        <v>18.02</v>
       </c>
       <c r="H108" t="n">
-        <v>20.49</v>
+        <v>17.75</v>
       </c>
       <c r="I108" t="n">
-        <v>20.72</v>
+        <v>18.16</v>
       </c>
       <c r="J108" t="n">
-        <v>20.25</v>
+        <v>17.42</v>
       </c>
       <c r="K108" t="n">
-        <v>20.78</v>
+        <v>18.02</v>
       </c>
       <c r="L108" t="n">
-        <v>20.92</v>
+        <v>18.32</v>
       </c>
       <c r="M108" t="n">
-        <v>20.83</v>
+        <v>18.24</v>
       </c>
       <c r="N108" t="n">
-        <v>20.47</v>
+        <v>17.9</v>
       </c>
       <c r="O108" t="n">
-        <v>20.45</v>
+        <v>17.95</v>
       </c>
       <c r="P108" t="n">
-        <v>21.06</v>
+        <v>18.49</v>
       </c>
     </row>
     <row r="109">
@@ -6498,52 +6498,52 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D109" t="n">
         <v>2003</v>
       </c>
       <c r="E109" t="n">
-        <v>21.2</v>
+        <v>18.55</v>
       </c>
       <c r="F109" t="n">
-        <v>21.38</v>
+        <v>18.72</v>
       </c>
       <c r="G109" t="n">
-        <v>21.18</v>
+        <v>18.37</v>
       </c>
       <c r="H109" t="n">
-        <v>20.97</v>
+        <v>18.31</v>
       </c>
       <c r="I109" t="n">
-        <v>20.85</v>
+        <v>18.3</v>
       </c>
       <c r="J109" t="n">
-        <v>20.06</v>
+        <v>17.21</v>
       </c>
       <c r="K109" t="n">
-        <v>20.43</v>
+        <v>17.62</v>
       </c>
       <c r="L109" t="n">
-        <v>20.49</v>
+        <v>17.82</v>
       </c>
       <c r="M109" t="n">
-        <v>20.58</v>
+        <v>17.88</v>
       </c>
       <c r="N109" t="n">
-        <v>20.23</v>
+        <v>17.55</v>
       </c>
       <c r="O109" t="n">
-        <v>20.28</v>
+        <v>17.56</v>
       </c>
       <c r="P109" t="n">
-        <v>20.52</v>
+        <v>17.84</v>
       </c>
     </row>
     <row r="110">
@@ -6554,52 +6554,52 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D110" t="n">
         <v>2004</v>
       </c>
       <c r="E110" t="n">
-        <v>20.37</v>
+        <v>17.61</v>
       </c>
       <c r="F110" t="n">
-        <v>20.87</v>
+        <v>18.2</v>
       </c>
       <c r="G110" t="n">
-        <v>21.32</v>
+        <v>18.76</v>
       </c>
       <c r="H110" t="n">
-        <v>20.77</v>
+        <v>18.09</v>
       </c>
       <c r="I110" t="n">
-        <v>20.36</v>
+        <v>17.7</v>
       </c>
       <c r="J110" t="n">
-        <v>20.5</v>
+        <v>17.92</v>
       </c>
       <c r="K110" t="n">
-        <v>20.34</v>
+        <v>17.37</v>
       </c>
       <c r="L110" t="n">
-        <v>20.79</v>
+        <v>18.16</v>
       </c>
       <c r="M110" t="n">
-        <v>20.15</v>
+        <v>17.28</v>
       </c>
       <c r="N110" t="n">
-        <v>20.19</v>
+        <v>17.35</v>
       </c>
       <c r="O110" t="n">
-        <v>19.95</v>
+        <v>17.45</v>
       </c>
       <c r="P110" t="n">
-        <v>20.27</v>
+        <v>17.64</v>
       </c>
     </row>
     <row r="111">
@@ -6610,52 +6610,52 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D111" t="n">
         <v>2005</v>
       </c>
       <c r="E111" t="n">
-        <v>20.57</v>
+        <v>17.82</v>
       </c>
       <c r="F111" t="n">
-        <v>20.71</v>
+        <v>18.21</v>
       </c>
       <c r="G111" t="n">
-        <v>21.43</v>
+        <v>18.57</v>
       </c>
       <c r="H111" t="n">
-        <v>21.36</v>
+        <v>18.8</v>
       </c>
       <c r="I111" t="n">
-        <v>20.67</v>
+        <v>17.95</v>
       </c>
       <c r="J111" t="n">
-        <v>20.92</v>
+        <v>18.05</v>
       </c>
       <c r="K111" t="n">
-        <v>21.07</v>
+        <v>18.26</v>
       </c>
       <c r="L111" t="n">
-        <v>20.95</v>
+        <v>18.22</v>
       </c>
       <c r="M111" t="n">
-        <v>20.87</v>
+        <v>18.23</v>
       </c>
       <c r="N111" t="n">
-        <v>20.06</v>
+        <v>17.3</v>
       </c>
       <c r="O111" t="n">
-        <v>19.87</v>
+        <v>17.35</v>
       </c>
       <c r="P111" t="n">
-        <v>20.04</v>
+        <v>17.25</v>
       </c>
     </row>
     <row r="112">
@@ -6666,52 +6666,52 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D112" t="n">
         <v>2006</v>
       </c>
       <c r="E112" t="n">
-        <v>20.34</v>
+        <v>17.63</v>
       </c>
       <c r="F112" t="n">
-        <v>20.78</v>
+        <v>18.11</v>
       </c>
       <c r="G112" t="n">
-        <v>20.58</v>
+        <v>17.72</v>
       </c>
       <c r="H112" t="n">
-        <v>20.57</v>
+        <v>17.89</v>
       </c>
       <c r="I112" t="n">
-        <v>20.49</v>
+        <v>17.84</v>
       </c>
       <c r="J112" t="n">
-        <v>20.41</v>
+        <v>17.61</v>
       </c>
       <c r="K112" t="n">
-        <v>20.87</v>
+        <v>18.12</v>
       </c>
       <c r="L112" t="n">
-        <v>20.9</v>
+        <v>18.22</v>
       </c>
       <c r="M112" t="n">
-        <v>20.79</v>
+        <v>18.14</v>
       </c>
       <c r="N112" t="n">
-        <v>20.65</v>
+        <v>18.09</v>
       </c>
       <c r="O112" t="n">
-        <v>20.33</v>
+        <v>17.76</v>
       </c>
       <c r="P112" t="n">
-        <v>20.63</v>
+        <v>17.94</v>
       </c>
     </row>
     <row r="113">
@@ -6722,52 +6722,52 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D113" t="n">
         <v>2007</v>
       </c>
       <c r="E113" t="n">
-        <v>20.54</v>
+        <v>18.01</v>
       </c>
       <c r="F113" t="n">
-        <v>20.94</v>
+        <v>18.44</v>
       </c>
       <c r="G113" t="n">
-        <v>21.03</v>
+        <v>18.17</v>
       </c>
       <c r="H113" t="n">
-        <v>20.78</v>
+        <v>17.95</v>
       </c>
       <c r="I113" t="n">
-        <v>20.57</v>
+        <v>17.8</v>
       </c>
       <c r="J113" t="n">
-        <v>20.49</v>
+        <v>17.7</v>
       </c>
       <c r="K113" t="n">
-        <v>20.79</v>
+        <v>17.92</v>
       </c>
       <c r="L113" t="n">
-        <v>20.37</v>
+        <v>17.48</v>
       </c>
       <c r="M113" t="n">
-        <v>20.36</v>
+        <v>17.77</v>
       </c>
       <c r="N113" t="n">
-        <v>19.73</v>
+        <v>17</v>
       </c>
       <c r="O113" t="n">
-        <v>19.98</v>
+        <v>17.21</v>
       </c>
       <c r="P113" t="n">
-        <v>20.39</v>
+        <v>17.49</v>
       </c>
     </row>
     <row r="114">
@@ -6778,52 +6778,52 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D114" t="n">
         <v>2008</v>
       </c>
       <c r="E114" t="n">
-        <v>20.33</v>
+        <v>17.52</v>
       </c>
       <c r="F114" t="n">
-        <v>20.4</v>
+        <v>17.62</v>
       </c>
       <c r="G114" t="n">
-        <v>20.38</v>
+        <v>17.52</v>
       </c>
       <c r="H114" t="n">
-        <v>20.56</v>
+        <v>17.74</v>
       </c>
       <c r="I114" t="n">
-        <v>20.07</v>
+        <v>17.25</v>
       </c>
       <c r="J114" t="n">
-        <v>20.24</v>
+        <v>17.45</v>
       </c>
       <c r="K114" t="n">
-        <v>20.25</v>
+        <v>17.32</v>
       </c>
       <c r="L114" t="n">
-        <v>20.24</v>
+        <v>17.34</v>
       </c>
       <c r="M114" t="n">
-        <v>20.48</v>
+        <v>17.69</v>
       </c>
       <c r="N114" t="n">
-        <v>20.01</v>
+        <v>17.39</v>
       </c>
       <c r="O114" t="n">
-        <v>19.9</v>
+        <v>17.35</v>
       </c>
       <c r="P114" t="n">
-        <v>20.02</v>
+        <v>17.28</v>
       </c>
     </row>
     <row r="115">
@@ -6834,52 +6834,52 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D115" t="n">
         <v>2009</v>
       </c>
       <c r="E115" t="n">
-        <v>20.35</v>
+        <v>17.62</v>
       </c>
       <c r="F115" t="n">
-        <v>20.33</v>
+        <v>17.59</v>
       </c>
       <c r="G115" t="n">
-        <v>19.96</v>
+        <v>16.98</v>
       </c>
       <c r="H115" t="n">
-        <v>20.95</v>
+        <v>18.39</v>
       </c>
       <c r="I115" t="n">
-        <v>20.7</v>
+        <v>18.15</v>
       </c>
       <c r="J115" t="n">
-        <v>20.71</v>
+        <v>18.13</v>
       </c>
       <c r="K115" t="n">
-        <v>21.09</v>
+        <v>18.53</v>
       </c>
       <c r="L115" t="n">
-        <v>21.36</v>
+        <v>18.84</v>
       </c>
       <c r="M115" t="n">
-        <v>21.39</v>
+        <v>19.02</v>
       </c>
       <c r="N115" t="n">
-        <v>20.78</v>
+        <v>18.38</v>
       </c>
       <c r="O115" t="n">
-        <v>21.11</v>
+        <v>18.62</v>
       </c>
       <c r="P115" t="n">
-        <v>21.08</v>
+        <v>18.46</v>
       </c>
     </row>
     <row r="116">
@@ -6890,52 +6890,52 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D116" t="n">
         <v>2010</v>
       </c>
       <c r="E116" t="n">
-        <v>21.18</v>
+        <v>18.81</v>
       </c>
       <c r="F116" t="n">
-        <v>21.46</v>
+        <v>18.96</v>
       </c>
       <c r="G116" t="n">
-        <v>22.1</v>
+        <v>19.61</v>
       </c>
       <c r="H116" t="n">
-        <v>21.28</v>
+        <v>18.71</v>
       </c>
       <c r="I116" t="n">
-        <v>21.06</v>
+        <v>18.51</v>
       </c>
       <c r="J116" t="n">
-        <v>20.56</v>
+        <v>17.87</v>
       </c>
       <c r="K116" t="n">
-        <v>20.51</v>
+        <v>17.66</v>
       </c>
       <c r="L116" t="n">
-        <v>20.67</v>
+        <v>17.99</v>
       </c>
       <c r="M116" t="n">
-        <v>20.34</v>
+        <v>17.71</v>
       </c>
       <c r="N116" t="n">
-        <v>20.27</v>
+        <v>17.75</v>
       </c>
       <c r="O116" t="n">
-        <v>19.65</v>
+        <v>17.09</v>
       </c>
       <c r="P116" t="n">
-        <v>19.84</v>
+        <v>17.09</v>
       </c>
     </row>
     <row r="117">
@@ -6946,52 +6946,52 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D117" t="n">
         <v>2011</v>
       </c>
       <c r="E117" t="n">
-        <v>20.4</v>
+        <v>17.72</v>
       </c>
       <c r="F117" t="n">
-        <v>20.44</v>
+        <v>17.66</v>
       </c>
       <c r="G117" t="n">
-        <v>20.24</v>
+        <v>17.43</v>
       </c>
       <c r="H117" t="n">
-        <v>20.33</v>
+        <v>17.62</v>
       </c>
       <c r="I117" t="n">
-        <v>20.52</v>
+        <v>17.91</v>
       </c>
       <c r="J117" t="n">
-        <v>20.9</v>
+        <v>18.26</v>
       </c>
       <c r="K117" t="n">
-        <v>20.93</v>
+        <v>18.03</v>
       </c>
       <c r="L117" t="n">
-        <v>20.96</v>
+        <v>18.28</v>
       </c>
       <c r="M117" t="n">
-        <v>20.92</v>
+        <v>18.33</v>
       </c>
       <c r="N117" t="n">
-        <v>19.87</v>
+        <v>17.21</v>
       </c>
       <c r="O117" t="n">
-        <v>20.19</v>
+        <v>17.66</v>
       </c>
       <c r="P117" t="n">
-        <v>20.23</v>
+        <v>17.46</v>
       </c>
     </row>
     <row r="118">
@@ -7002,52 +7002,52 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D118" t="n">
         <v>2012</v>
       </c>
       <c r="E118" t="n">
-        <v>20.34</v>
+        <v>17.58</v>
       </c>
       <c r="F118" t="n">
-        <v>20.6</v>
+        <v>17.82</v>
       </c>
       <c r="G118" t="n">
-        <v>20.93</v>
+        <v>18.12</v>
       </c>
       <c r="H118" t="n">
-        <v>20.59</v>
+        <v>17.8</v>
       </c>
       <c r="I118" t="n">
-        <v>21.03</v>
+        <v>18.21</v>
       </c>
       <c r="J118" t="n">
-        <v>21.14</v>
+        <v>18.4</v>
       </c>
       <c r="K118" t="n">
-        <v>21.33</v>
+        <v>18.57</v>
       </c>
       <c r="L118" t="n">
-        <v>20.98</v>
+        <v>18.32</v>
       </c>
       <c r="M118" t="n">
-        <v>21.35</v>
+        <v>18.77</v>
       </c>
       <c r="N118" t="n">
-        <v>20.7</v>
+        <v>18.1</v>
       </c>
       <c r="O118" t="n">
-        <v>20.4</v>
+        <v>17.9</v>
       </c>
       <c r="P118" t="n">
-        <v>20.8</v>
+        <v>18.28</v>
       </c>
     </row>
     <row r="119">
@@ -7058,52 +7058,52 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D119" t="n">
         <v>2013</v>
       </c>
       <c r="E119" t="n">
-        <v>21.26</v>
+        <v>18.9</v>
       </c>
       <c r="F119" t="n">
-        <v>20.99</v>
+        <v>18.26</v>
       </c>
       <c r="G119" t="n">
-        <v>21.46</v>
+        <v>18.72</v>
       </c>
       <c r="H119" t="n">
-        <v>21.47</v>
+        <v>18.9</v>
       </c>
       <c r="I119" t="n">
-        <v>20.49</v>
+        <v>17.72</v>
       </c>
       <c r="J119" t="n">
-        <v>21.09</v>
+        <v>18.51</v>
       </c>
       <c r="K119" t="n">
-        <v>21.19</v>
+        <v>18.37</v>
       </c>
       <c r="L119" t="n">
-        <v>20.77</v>
+        <v>18.03</v>
       </c>
       <c r="M119" t="n">
-        <v>21.15</v>
+        <v>18.64</v>
       </c>
       <c r="N119" t="n">
-        <v>20.86</v>
+        <v>18.29</v>
       </c>
       <c r="O119" t="n">
-        <v>20.65</v>
+        <v>18.02</v>
       </c>
       <c r="P119" t="n">
-        <v>20.73</v>
+        <v>18.04</v>
       </c>
     </row>
     <row r="120">
@@ -7114,52 +7114,52 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D120" t="n">
         <v>2014</v>
       </c>
       <c r="E120" t="n">
-        <v>21.03</v>
+        <v>18.32</v>
       </c>
       <c r="F120" t="n">
-        <v>21.08</v>
+        <v>18.41</v>
       </c>
       <c r="G120" t="n">
-        <v>21.27</v>
+        <v>18.47</v>
       </c>
       <c r="H120" t="n">
-        <v>21.56</v>
+        <v>18.94</v>
       </c>
       <c r="I120" t="n">
-        <v>21</v>
+        <v>18.31</v>
       </c>
       <c r="J120" t="n">
-        <v>21.51</v>
+        <v>18.8</v>
       </c>
       <c r="K120" t="n">
-        <v>22.04</v>
+        <v>19.41</v>
       </c>
       <c r="L120" t="n">
-        <v>21.54</v>
+        <v>18.82</v>
       </c>
       <c r="M120" t="n">
-        <v>21.37</v>
+        <v>18.83</v>
       </c>
       <c r="N120" t="n">
-        <v>20.82</v>
+        <v>18.2</v>
       </c>
       <c r="O120" t="n">
-        <v>20.9</v>
+        <v>18.35</v>
       </c>
       <c r="P120" t="n">
-        <v>21.14</v>
+        <v>18.53</v>
       </c>
     </row>
     <row r="121">
@@ -7170,52 +7170,52 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D121" t="n">
         <v>2015</v>
       </c>
       <c r="E121" t="n">
-        <v>21.25</v>
+        <v>18.66</v>
       </c>
       <c r="F121" t="n">
-        <v>21.48</v>
+        <v>18.81</v>
       </c>
       <c r="G121" t="n">
-        <v>21.25</v>
+        <v>18.43</v>
       </c>
       <c r="H121" t="n">
-        <v>21.33</v>
+        <v>18.7</v>
       </c>
       <c r="I121" t="n">
-        <v>21.63</v>
+        <v>19.02</v>
       </c>
       <c r="J121" t="n">
-        <v>21.25</v>
+        <v>18.7</v>
       </c>
       <c r="K121" t="n">
-        <v>21.84</v>
+        <v>19.04</v>
       </c>
       <c r="L121" t="n">
-        <v>22.05</v>
+        <v>19.32</v>
       </c>
       <c r="M121" t="n">
-        <v>21.81</v>
+        <v>19.38</v>
       </c>
       <c r="N121" t="n">
-        <v>21.62</v>
+        <v>18.89</v>
       </c>
       <c r="O121" t="n">
-        <v>21.19</v>
+        <v>18.62</v>
       </c>
       <c r="P121" t="n">
-        <v>21.79</v>
+        <v>18.93</v>
       </c>
     </row>
     <row r="122">
@@ -7226,52 +7226,52 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D122" t="n">
         <v>2016</v>
       </c>
       <c r="E122" t="n">
-        <v>21.86</v>
+        <v>19.21</v>
       </c>
       <c r="F122" t="n">
-        <v>21.81</v>
+        <v>19.41</v>
       </c>
       <c r="G122" t="n">
-        <v>21.42</v>
+        <v>18.78</v>
       </c>
       <c r="H122" t="n">
-        <v>21.82</v>
+        <v>19.11</v>
       </c>
       <c r="I122" t="n">
-        <v>21.73</v>
+        <v>19.05</v>
       </c>
       <c r="J122" t="n">
-        <v>21.36</v>
+        <v>18.56</v>
       </c>
       <c r="K122" t="n">
-        <v>21.28</v>
+        <v>18.48</v>
       </c>
       <c r="L122" t="n">
-        <v>21.89</v>
+        <v>19.24</v>
       </c>
       <c r="M122" t="n">
-        <v>21.24</v>
+        <v>18.44</v>
       </c>
       <c r="N122" t="n">
-        <v>20.77</v>
+        <v>18.11</v>
       </c>
       <c r="O122" t="n">
-        <v>20.36</v>
+        <v>17.88</v>
       </c>
       <c r="P122" t="n">
-        <v>20.62</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="123">
@@ -7282,52 +7282,52 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D123" t="n">
         <v>2017</v>
       </c>
       <c r="E123" t="n">
-        <v>20.25</v>
+        <v>17.71</v>
       </c>
       <c r="F123" t="n">
-        <v>20.76</v>
+        <v>18.21</v>
       </c>
       <c r="G123" t="n">
-        <v>20.31</v>
+        <v>17.72</v>
       </c>
       <c r="H123" t="n">
-        <v>21.2</v>
+        <v>18.69</v>
       </c>
       <c r="I123" t="n">
-        <v>20.98</v>
+        <v>18.21</v>
       </c>
       <c r="J123" t="n">
-        <v>20.76</v>
+        <v>18.07</v>
       </c>
       <c r="K123" t="n">
-        <v>21.07</v>
+        <v>18.42</v>
       </c>
       <c r="L123" t="n">
-        <v>20.54</v>
+        <v>18.01</v>
       </c>
       <c r="M123" t="n">
-        <v>21.3</v>
+        <v>18.77</v>
       </c>
       <c r="N123" t="n">
-        <v>20.68</v>
+        <v>18.14</v>
       </c>
       <c r="O123" t="n">
-        <v>20.47</v>
+        <v>18.05</v>
       </c>
       <c r="P123" t="n">
-        <v>20.35</v>
+        <v>17.78</v>
       </c>
     </row>
     <row r="124">
@@ -7338,52 +7338,52 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D124" t="n">
         <v>2018</v>
       </c>
       <c r="E124" t="n">
-        <v>20.25</v>
+        <v>17.71</v>
       </c>
       <c r="F124" t="n">
-        <v>20.57</v>
+        <v>18.01</v>
       </c>
       <c r="G124" t="n">
-        <v>21</v>
+        <v>18.47</v>
       </c>
       <c r="H124" t="n">
-        <v>20.41</v>
+        <v>17.89</v>
       </c>
       <c r="I124" t="n">
-        <v>20.25</v>
+        <v>17.75</v>
       </c>
       <c r="J124" t="n">
-        <v>20.61</v>
+        <v>18.1</v>
       </c>
       <c r="K124" t="n">
-        <v>20.86</v>
+        <v>18.22</v>
       </c>
       <c r="L124" t="n">
-        <v>20.98</v>
+        <v>18.42</v>
       </c>
       <c r="M124" t="n">
-        <v>20.81</v>
+        <v>18.33</v>
       </c>
       <c r="N124" t="n">
-        <v>20.41</v>
+        <v>17.9</v>
       </c>
       <c r="O124" t="n">
-        <v>20.4</v>
+        <v>17.96</v>
       </c>
       <c r="P124" t="n">
-        <v>20.77</v>
+        <v>18.32</v>
       </c>
     </row>
     <row r="125">
@@ -7394,52 +7394,52 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D125" t="n">
         <v>2019</v>
       </c>
       <c r="E125" t="n">
-        <v>20.95</v>
+        <v>18.41</v>
       </c>
       <c r="F125" t="n">
-        <v>21.47</v>
+        <v>18.91</v>
       </c>
       <c r="G125" t="n">
-        <v>21.02</v>
+        <v>18.42</v>
       </c>
       <c r="H125" t="n">
-        <v>21.21</v>
+        <v>18.7</v>
       </c>
       <c r="I125" t="n">
-        <v>20.86</v>
+        <v>18.31</v>
       </c>
       <c r="J125" t="n">
-        <v>21.17</v>
+        <v>18.65</v>
       </c>
       <c r="K125" t="n">
-        <v>21.26</v>
+        <v>18.66</v>
       </c>
       <c r="L125" t="n">
-        <v>21.64</v>
+        <v>19.11</v>
       </c>
       <c r="M125" t="n">
-        <v>21.31</v>
+        <v>18.83</v>
       </c>
       <c r="N125" t="n">
-        <v>20.39</v>
+        <v>17.89</v>
       </c>
       <c r="O125" t="n">
-        <v>20.79</v>
+        <v>18.3</v>
       </c>
       <c r="P125" t="n">
-        <v>21.01</v>
+        <v>18.43</v>
       </c>
     </row>
     <row r="126">
@@ -7450,52 +7450,52 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D126" t="n">
         <v>2020</v>
       </c>
       <c r="E126" t="n">
-        <v>21.34</v>
+        <v>18.8</v>
       </c>
       <c r="F126" t="n">
-        <v>21.92</v>
+        <v>19.34</v>
       </c>
       <c r="G126" t="n">
-        <v>21.7</v>
+        <v>19.06</v>
       </c>
       <c r="H126" t="n">
-        <v>21.63</v>
+        <v>19.09</v>
       </c>
       <c r="I126" t="n">
-        <v>21.14</v>
+        <v>18.54</v>
       </c>
       <c r="J126" t="n">
-        <v>20.67</v>
+        <v>18.15</v>
       </c>
       <c r="K126" t="n">
-        <v>20.61</v>
+        <v>18.02</v>
       </c>
       <c r="L126" t="n">
-        <v>20.64</v>
+        <v>18.12</v>
       </c>
       <c r="M126" t="n">
-        <v>20.52</v>
+        <v>18.09</v>
       </c>
       <c r="N126" t="n">
-        <v>20.6</v>
+        <v>18.09</v>
       </c>
       <c r="O126" t="n">
-        <v>20.19</v>
+        <v>17.75</v>
       </c>
       <c r="P126" t="n">
-        <v>20.35</v>
+        <v>17.83</v>
       </c>
     </row>
     <row r="127">
@@ -7506,52 +7506,52 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D127" t="n">
         <v>2021</v>
       </c>
       <c r="E127" t="n">
-        <v>20.63</v>
+        <v>18.04</v>
       </c>
       <c r="F127" t="n">
-        <v>20.83</v>
+        <v>18.16</v>
       </c>
       <c r="G127" t="n">
-        <v>20.03</v>
+        <v>17.42</v>
       </c>
       <c r="H127" t="n">
-        <v>20.62</v>
+        <v>18.1</v>
       </c>
       <c r="I127" t="n">
-        <v>20.57</v>
+        <v>18</v>
       </c>
       <c r="J127" t="n">
-        <v>20.01</v>
+        <v>17.41</v>
       </c>
       <c r="K127" t="n">
-        <v>20.66</v>
+        <v>18.02</v>
       </c>
       <c r="L127" t="n">
-        <v>19.97</v>
+        <v>17.43</v>
       </c>
       <c r="M127" t="n">
-        <v>20.42</v>
+        <v>17.93</v>
       </c>
       <c r="N127" t="n">
-        <v>20.22</v>
+        <v>17.7</v>
       </c>
       <c r="O127" t="n">
-        <v>20</v>
+        <v>17.56</v>
       </c>
       <c r="P127" t="n">
-        <v>20.37</v>
+        <v>17.85</v>
       </c>
     </row>
     <row r="128">
@@ -7562,52 +7562,52 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D128" t="n">
         <v>2022</v>
       </c>
       <c r="E128" t="n">
-        <v>20.26</v>
+        <v>17.72</v>
       </c>
       <c r="F128" t="n">
-        <v>20.19</v>
+        <v>17.57</v>
       </c>
       <c r="G128" t="n">
-        <v>20.14</v>
+        <v>17.47</v>
       </c>
       <c r="H128" t="n">
-        <v>20.41</v>
+        <v>17.9</v>
       </c>
       <c r="I128" t="n">
-        <v>20.44</v>
+        <v>17.9</v>
       </c>
       <c r="J128" t="n">
-        <v>19.18</v>
+        <v>16.61</v>
       </c>
       <c r="K128" t="n">
-        <v>20.17</v>
+        <v>17.52</v>
       </c>
       <c r="L128" t="n">
-        <v>20.19</v>
+        <v>17.68</v>
       </c>
       <c r="M128" t="n">
-        <v>20.02</v>
+        <v>17.53</v>
       </c>
       <c r="N128" t="n">
-        <v>20.17</v>
+        <v>17.74</v>
       </c>
       <c r="O128" t="n">
-        <v>19.6</v>
+        <v>17.21</v>
       </c>
       <c r="P128" t="n">
-        <v>19.97</v>
+        <v>17.43</v>
       </c>
     </row>
     <row r="129">
@@ -7618,52 +7618,52 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D129" t="n">
         <v>2023</v>
       </c>
       <c r="E129" t="n">
-        <v>19.78</v>
+        <v>17.22</v>
       </c>
       <c r="F129" t="n">
-        <v>20.69</v>
+        <v>18.11</v>
       </c>
       <c r="G129" t="n">
-        <v>20.22</v>
+        <v>17.57</v>
       </c>
       <c r="H129" t="n">
-        <v>20.41</v>
+        <v>17.9</v>
       </c>
       <c r="I129" t="n">
-        <v>21.34</v>
+        <v>18.61</v>
       </c>
       <c r="J129" t="n">
-        <v>21.18</v>
+        <v>18.57</v>
       </c>
       <c r="K129" t="n">
-        <v>21.32</v>
+        <v>18.62</v>
       </c>
       <c r="L129" t="n">
-        <v>21.41</v>
+        <v>18.82</v>
       </c>
       <c r="M129" t="n">
-        <v>21.41</v>
+        <v>18.87</v>
       </c>
       <c r="N129" t="n">
-        <v>20.9</v>
+        <v>18.44</v>
       </c>
       <c r="O129" t="n">
-        <v>20.79</v>
+        <v>18.35</v>
       </c>
       <c r="P129" t="n">
-        <v>21.08</v>
+        <v>18.48</v>
       </c>
     </row>
     <row r="130">
@@ -7674,52 +7674,52 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D130" t="n">
         <v>2024</v>
       </c>
       <c r="E130" t="n">
-        <v>21.61</v>
+        <v>19.06</v>
       </c>
       <c r="F130" t="n">
-        <v>22.07</v>
+        <v>19.5</v>
       </c>
       <c r="G130" t="n">
-        <v>21.39</v>
+        <v>18.81</v>
       </c>
       <c r="H130" t="n">
-        <v>21.51</v>
+        <v>19</v>
       </c>
       <c r="I130" t="n">
-        <v>21.45</v>
+        <v>18.85</v>
       </c>
       <c r="J130" t="n">
-        <v>20.41</v>
+        <v>17.81</v>
       </c>
       <c r="K130" t="n">
-        <v>21.36</v>
+        <v>18.77</v>
       </c>
       <c r="L130" t="n">
-        <v>21.29</v>
+        <v>18.77</v>
       </c>
       <c r="M130" t="n">
-        <v>21.72</v>
+        <v>19.24</v>
       </c>
       <c r="N130" t="n">
-        <v>20.69</v>
+        <v>18.19</v>
       </c>
       <c r="O130" t="n">
-        <v>20.41</v>
+        <v>18.02</v>
       </c>
       <c r="P130" t="n">
-        <v>20.91</v>
+        <v>18.39</v>
       </c>
     </row>
     <row r="131">
@@ -7730,51 +7730,1507 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>COL.57959</t>
+          <t>COL.57958</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Risaralda</t>
+          <t>Quindio</t>
         </is>
       </c>
       <c r="D131" t="n">
         <v>2025</v>
       </c>
       <c r="E131" t="n">
+        <v>18.41</v>
+      </c>
+      <c r="F131" t="n">
+        <v>18.12</v>
+      </c>
+      <c r="G131" t="n">
+        <v>18.42</v>
+      </c>
+      <c r="H131" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="I131" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="J131" t="n">
+        <v>18.01</v>
+      </c>
+      <c r="K131" t="n">
+        <v>18.96</v>
+      </c>
+      <c r="L131" t="n">
+        <v>18.72</v>
+      </c>
+      <c r="M131" t="n">
+        <v>18.84</v>
+      </c>
+      <c r="N131" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="O131" t="n">
+        <v>18.55</v>
+      </c>
+      <c r="P131" t="n">
+        <v>18.33</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E132" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="F132" t="n">
+        <v>19.95</v>
+      </c>
+      <c r="G132" t="n">
+        <v>20.09</v>
+      </c>
+      <c r="H132" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="I132" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="J132" t="n">
+        <v>19.83</v>
+      </c>
+      <c r="K132" t="n">
+        <v>19.85</v>
+      </c>
+      <c r="L132" t="n">
+        <v>20.36</v>
+      </c>
+      <c r="M132" t="n">
+        <v>19.81</v>
+      </c>
+      <c r="N132" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="O132" t="n">
+        <v>19.81</v>
+      </c>
+      <c r="P132" t="n">
+        <v>20.19</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E133" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="F133" t="n">
+        <v>20.16</v>
+      </c>
+      <c r="G133" t="n">
+        <v>20.61</v>
+      </c>
+      <c r="H133" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="I133" t="n">
+        <v>20.55</v>
+      </c>
+      <c r="J133" t="n">
+        <v>20.18</v>
+      </c>
+      <c r="K133" t="n">
+        <v>20.59</v>
+      </c>
+      <c r="L133" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="M133" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="N133" t="n">
+        <v>20.44</v>
+      </c>
+      <c r="O133" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="P133" t="n">
+        <v>20.71</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E134" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="F134" t="n">
+        <v>20.77</v>
+      </c>
+      <c r="G134" t="n">
+        <v>20.73</v>
+      </c>
+      <c r="H134" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="I134" t="n">
+        <v>20.72</v>
+      </c>
+      <c r="J134" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="K134" t="n">
+        <v>20.78</v>
+      </c>
+      <c r="L134" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="M134" t="n">
+        <v>20.83</v>
+      </c>
+      <c r="N134" t="n">
+        <v>20.47</v>
+      </c>
+      <c r="O134" t="n">
+        <v>20.45</v>
+      </c>
+      <c r="P134" t="n">
+        <v>21.06</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E135" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="F135" t="n">
+        <v>21.38</v>
+      </c>
+      <c r="G135" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="H135" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="I135" t="n">
+        <v>20.85</v>
+      </c>
+      <c r="J135" t="n">
+        <v>20.06</v>
+      </c>
+      <c r="K135" t="n">
+        <v>20.43</v>
+      </c>
+      <c r="L135" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="M135" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="N135" t="n">
+        <v>20.23</v>
+      </c>
+      <c r="O135" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="P135" t="n">
+        <v>20.52</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E136" t="n">
+        <v>20.37</v>
+      </c>
+      <c r="F136" t="n">
+        <v>20.87</v>
+      </c>
+      <c r="G136" t="n">
+        <v>21.32</v>
+      </c>
+      <c r="H136" t="n">
+        <v>20.77</v>
+      </c>
+      <c r="I136" t="n">
+        <v>20.36</v>
+      </c>
+      <c r="J136" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="K136" t="n">
+        <v>20.34</v>
+      </c>
+      <c r="L136" t="n">
+        <v>20.79</v>
+      </c>
+      <c r="M136" t="n">
+        <v>20.15</v>
+      </c>
+      <c r="N136" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="O136" t="n">
+        <v>19.95</v>
+      </c>
+      <c r="P136" t="n">
+        <v>20.27</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E137" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="F137" t="n">
+        <v>20.71</v>
+      </c>
+      <c r="G137" t="n">
+        <v>21.43</v>
+      </c>
+      <c r="H137" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="I137" t="n">
+        <v>20.67</v>
+      </c>
+      <c r="J137" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="K137" t="n">
+        <v>21.07</v>
+      </c>
+      <c r="L137" t="n">
+        <v>20.95</v>
+      </c>
+      <c r="M137" t="n">
+        <v>20.87</v>
+      </c>
+      <c r="N137" t="n">
+        <v>20.06</v>
+      </c>
+      <c r="O137" t="n">
+        <v>19.87</v>
+      </c>
+      <c r="P137" t="n">
+        <v>20.04</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E138" t="n">
+        <v>20.34</v>
+      </c>
+      <c r="F138" t="n">
+        <v>20.78</v>
+      </c>
+      <c r="G138" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="H138" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="I138" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="J138" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="K138" t="n">
+        <v>20.87</v>
+      </c>
+      <c r="L138" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="M138" t="n">
+        <v>20.79</v>
+      </c>
+      <c r="N138" t="n">
+        <v>20.65</v>
+      </c>
+      <c r="O138" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="P138" t="n">
+        <v>20.63</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E139" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="F139" t="n">
+        <v>20.94</v>
+      </c>
+      <c r="G139" t="n">
+        <v>21.03</v>
+      </c>
+      <c r="H139" t="n">
+        <v>20.78</v>
+      </c>
+      <c r="I139" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="J139" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="K139" t="n">
+        <v>20.79</v>
+      </c>
+      <c r="L139" t="n">
+        <v>20.37</v>
+      </c>
+      <c r="M139" t="n">
+        <v>20.36</v>
+      </c>
+      <c r="N139" t="n">
+        <v>19.73</v>
+      </c>
+      <c r="O139" t="n">
+        <v>19.98</v>
+      </c>
+      <c r="P139" t="n">
+        <v>20.39</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E140" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="F140" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G140" t="n">
+        <v>20.38</v>
+      </c>
+      <c r="H140" t="n">
+        <v>20.56</v>
+      </c>
+      <c r="I140" t="n">
+        <v>20.07</v>
+      </c>
+      <c r="J140" t="n">
+        <v>20.24</v>
+      </c>
+      <c r="K140" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="L140" t="n">
+        <v>20.24</v>
+      </c>
+      <c r="M140" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="N140" t="n">
+        <v>20.01</v>
+      </c>
+      <c r="O140" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="P140" t="n">
+        <v>20.02</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E141" t="n">
+        <v>20.35</v>
+      </c>
+      <c r="F141" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="G141" t="n">
+        <v>19.96</v>
+      </c>
+      <c r="H141" t="n">
+        <v>20.95</v>
+      </c>
+      <c r="I141" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="J141" t="n">
+        <v>20.71</v>
+      </c>
+      <c r="K141" t="n">
+        <v>21.09</v>
+      </c>
+      <c r="L141" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="M141" t="n">
+        <v>21.39</v>
+      </c>
+      <c r="N141" t="n">
+        <v>20.78</v>
+      </c>
+      <c r="O141" t="n">
+        <v>21.11</v>
+      </c>
+      <c r="P141" t="n">
+        <v>21.08</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E142" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="F142" t="n">
+        <v>21.46</v>
+      </c>
+      <c r="G142" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="H142" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="I142" t="n">
+        <v>21.06</v>
+      </c>
+      <c r="J142" t="n">
+        <v>20.56</v>
+      </c>
+      <c r="K142" t="n">
+        <v>20.51</v>
+      </c>
+      <c r="L142" t="n">
+        <v>20.67</v>
+      </c>
+      <c r="M142" t="n">
+        <v>20.34</v>
+      </c>
+      <c r="N142" t="n">
+        <v>20.27</v>
+      </c>
+      <c r="O142" t="n">
+        <v>19.65</v>
+      </c>
+      <c r="P142" t="n">
+        <v>19.84</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E143" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="F143" t="n">
+        <v>20.44</v>
+      </c>
+      <c r="G143" t="n">
+        <v>20.24</v>
+      </c>
+      <c r="H143" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="I143" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="J143" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="K143" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="L143" t="n">
+        <v>20.96</v>
+      </c>
+      <c r="M143" t="n">
+        <v>20.92</v>
+      </c>
+      <c r="N143" t="n">
+        <v>19.87</v>
+      </c>
+      <c r="O143" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="P143" t="n">
+        <v>20.23</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E144" t="n">
+        <v>20.34</v>
+      </c>
+      <c r="F144" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G144" t="n">
+        <v>20.93</v>
+      </c>
+      <c r="H144" t="n">
+        <v>20.59</v>
+      </c>
+      <c r="I144" t="n">
+        <v>21.03</v>
+      </c>
+      <c r="J144" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="K144" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="L144" t="n">
+        <v>20.98</v>
+      </c>
+      <c r="M144" t="n">
+        <v>21.35</v>
+      </c>
+      <c r="N144" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="O144" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="P144" t="n">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E145" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="F145" t="n">
         <v>20.99</v>
       </c>
-      <c r="F131" t="n">
+      <c r="G145" t="n">
+        <v>21.46</v>
+      </c>
+      <c r="H145" t="n">
+        <v>21.47</v>
+      </c>
+      <c r="I145" t="n">
+        <v>20.49</v>
+      </c>
+      <c r="J145" t="n">
+        <v>21.09</v>
+      </c>
+      <c r="K145" t="n">
+        <v>21.19</v>
+      </c>
+      <c r="L145" t="n">
+        <v>20.77</v>
+      </c>
+      <c r="M145" t="n">
+        <v>21.15</v>
+      </c>
+      <c r="N145" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="O145" t="n">
+        <v>20.65</v>
+      </c>
+      <c r="P145" t="n">
+        <v>20.73</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E146" t="n">
+        <v>21.03</v>
+      </c>
+      <c r="F146" t="n">
+        <v>21.08</v>
+      </c>
+      <c r="G146" t="n">
+        <v>21.27</v>
+      </c>
+      <c r="H146" t="n">
+        <v>21.56</v>
+      </c>
+      <c r="I146" t="n">
+        <v>21</v>
+      </c>
+      <c r="J146" t="n">
+        <v>21.51</v>
+      </c>
+      <c r="K146" t="n">
+        <v>22.04</v>
+      </c>
+      <c r="L146" t="n">
+        <v>21.54</v>
+      </c>
+      <c r="M146" t="n">
+        <v>21.37</v>
+      </c>
+      <c r="N146" t="n">
+        <v>20.82</v>
+      </c>
+      <c r="O146" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="P146" t="n">
+        <v>21.14</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E147" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="F147" t="n">
+        <v>21.48</v>
+      </c>
+      <c r="G147" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="H147" t="n">
+        <v>21.33</v>
+      </c>
+      <c r="I147" t="n">
+        <v>21.63</v>
+      </c>
+      <c r="J147" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="K147" t="n">
+        <v>21.84</v>
+      </c>
+      <c r="L147" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="M147" t="n">
+        <v>21.81</v>
+      </c>
+      <c r="N147" t="n">
+        <v>21.62</v>
+      </c>
+      <c r="O147" t="n">
+        <v>21.19</v>
+      </c>
+      <c r="P147" t="n">
+        <v>21.79</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E148" t="n">
+        <v>21.86</v>
+      </c>
+      <c r="F148" t="n">
+        <v>21.81</v>
+      </c>
+      <c r="G148" t="n">
+        <v>21.42</v>
+      </c>
+      <c r="H148" t="n">
+        <v>21.82</v>
+      </c>
+      <c r="I148" t="n">
+        <v>21.73</v>
+      </c>
+      <c r="J148" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="K148" t="n">
+        <v>21.28</v>
+      </c>
+      <c r="L148" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="M148" t="n">
+        <v>21.24</v>
+      </c>
+      <c r="N148" t="n">
+        <v>20.77</v>
+      </c>
+      <c r="O148" t="n">
+        <v>20.36</v>
+      </c>
+      <c r="P148" t="n">
+        <v>20.62</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E149" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="F149" t="n">
+        <v>20.76</v>
+      </c>
+      <c r="G149" t="n">
+        <v>20.31</v>
+      </c>
+      <c r="H149" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="I149" t="n">
+        <v>20.98</v>
+      </c>
+      <c r="J149" t="n">
+        <v>20.76</v>
+      </c>
+      <c r="K149" t="n">
+        <v>21.07</v>
+      </c>
+      <c r="L149" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="M149" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="N149" t="n">
         <v>20.68</v>
       </c>
-      <c r="G131" t="n">
+      <c r="O149" t="n">
+        <v>20.47</v>
+      </c>
+      <c r="P149" t="n">
+        <v>20.35</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E150" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="F150" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="G150" t="n">
+        <v>21</v>
+      </c>
+      <c r="H150" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="I150" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="J150" t="n">
+        <v>20.61</v>
+      </c>
+      <c r="K150" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="L150" t="n">
+        <v>20.98</v>
+      </c>
+      <c r="M150" t="n">
+        <v>20.81</v>
+      </c>
+      <c r="N150" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="O150" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="P150" t="n">
+        <v>20.77</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E151" t="n">
+        <v>20.95</v>
+      </c>
+      <c r="F151" t="n">
+        <v>21.47</v>
+      </c>
+      <c r="G151" t="n">
+        <v>21.02</v>
+      </c>
+      <c r="H151" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="I151" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="J151" t="n">
+        <v>21.17</v>
+      </c>
+      <c r="K151" t="n">
+        <v>21.26</v>
+      </c>
+      <c r="L151" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="M151" t="n">
+        <v>21.31</v>
+      </c>
+      <c r="N151" t="n">
+        <v>20.39</v>
+      </c>
+      <c r="O151" t="n">
+        <v>20.79</v>
+      </c>
+      <c r="P151" t="n">
+        <v>21.01</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E152" t="n">
+        <v>21.34</v>
+      </c>
+      <c r="F152" t="n">
+        <v>21.92</v>
+      </c>
+      <c r="G152" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="H152" t="n">
+        <v>21.63</v>
+      </c>
+      <c r="I152" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="J152" t="n">
+        <v>20.67</v>
+      </c>
+      <c r="K152" t="n">
+        <v>20.61</v>
+      </c>
+      <c r="L152" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="M152" t="n">
+        <v>20.52</v>
+      </c>
+      <c r="N152" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="O152" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="P152" t="n">
+        <v>20.35</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E153" t="n">
+        <v>20.63</v>
+      </c>
+      <c r="F153" t="n">
+        <v>20.83</v>
+      </c>
+      <c r="G153" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="H153" t="n">
+        <v>20.62</v>
+      </c>
+      <c r="I153" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="J153" t="n">
+        <v>20.01</v>
+      </c>
+      <c r="K153" t="n">
+        <v>20.66</v>
+      </c>
+      <c r="L153" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="M153" t="n">
+        <v>20.42</v>
+      </c>
+      <c r="N153" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="O153" t="n">
+        <v>20</v>
+      </c>
+      <c r="P153" t="n">
+        <v>20.37</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E154" t="n">
+        <v>20.26</v>
+      </c>
+      <c r="F154" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="G154" t="n">
+        <v>20.14</v>
+      </c>
+      <c r="H154" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="I154" t="n">
+        <v>20.44</v>
+      </c>
+      <c r="J154" t="n">
+        <v>19.18</v>
+      </c>
+      <c r="K154" t="n">
+        <v>20.17</v>
+      </c>
+      <c r="L154" t="n">
+        <v>20.19</v>
+      </c>
+      <c r="M154" t="n">
+        <v>20.02</v>
+      </c>
+      <c r="N154" t="n">
+        <v>20.17</v>
+      </c>
+      <c r="O154" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="P154" t="n">
+        <v>19.97</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E155" t="n">
+        <v>19.78</v>
+      </c>
+      <c r="F155" t="n">
+        <v>20.69</v>
+      </c>
+      <c r="G155" t="n">
+        <v>20.22</v>
+      </c>
+      <c r="H155" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="I155" t="n">
+        <v>21.34</v>
+      </c>
+      <c r="J155" t="n">
+        <v>21.18</v>
+      </c>
+      <c r="K155" t="n">
+        <v>21.32</v>
+      </c>
+      <c r="L155" t="n">
+        <v>21.41</v>
+      </c>
+      <c r="M155" t="n">
+        <v>21.41</v>
+      </c>
+      <c r="N155" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="O155" t="n">
+        <v>20.79</v>
+      </c>
+      <c r="P155" t="n">
+        <v>21.08</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E156" t="n">
+        <v>21.61</v>
+      </c>
+      <c r="F156" t="n">
+        <v>22.07</v>
+      </c>
+      <c r="G156" t="n">
+        <v>21.39</v>
+      </c>
+      <c r="H156" t="n">
+        <v>21.51</v>
+      </c>
+      <c r="I156" t="n">
+        <v>21.45</v>
+      </c>
+      <c r="J156" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="K156" t="n">
+        <v>21.36</v>
+      </c>
+      <c r="L156" t="n">
+        <v>21.29</v>
+      </c>
+      <c r="M156" t="n">
+        <v>21.72</v>
+      </c>
+      <c r="N156" t="n">
+        <v>20.69</v>
+      </c>
+      <c r="O156" t="n">
+        <v>20.41</v>
+      </c>
+      <c r="P156" t="n">
+        <v>20.91</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>COL.57959</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E157" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F157" t="n">
+        <v>20.68</v>
+      </c>
+      <c r="G157" t="n">
         <v>21.03</v>
       </c>
-      <c r="H131" t="n">
+      <c r="H157" t="n">
         <v>21.37</v>
       </c>
-      <c r="I131" t="n">
+      <c r="I157" t="n">
         <v>21.15</v>
       </c>
-      <c r="J131" t="n">
+      <c r="J157" t="n">
         <v>20.61</v>
       </c>
-      <c r="K131" t="n">
+      <c r="K157" t="n">
         <v>21.55</v>
       </c>
-      <c r="L131" t="n">
+      <c r="L157" t="n">
         <v>21.33</v>
       </c>
-      <c r="M131" t="n">
+      <c r="M157" t="n">
         <v>21.38</v>
       </c>
-      <c r="N131" t="n">
+      <c r="N157" t="n">
         <v>20.77</v>
       </c>
-      <c r="O131" t="n">
+      <c r="O157" t="n">
         <v>20.99</v>
       </c>
-      <c r="P131" t="n">
+      <c r="P157" t="n">
         <v>20.9</v>
       </c>
     </row>

</xml_diff>